<commit_message>
Test quiz round update with Excel
</commit_message>
<xml_diff>
--- a/QuizSettings.xlsx
+++ b/QuizSettings.xlsx
@@ -1,11 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30327"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6C329D2D-B3E9-4563-A84D-2DB2372B69CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cafnzholding-my.sharepoint.com/personal/thom_van_dusschoten_synerlogic_nl/Documents/Documenten/GitHub/Sustainability-quiz/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="1" documentId="8_{6C329D2D-B3E9-4563-A84D-2DB2372B69CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{084077E7-7CBA-4869-8D62-5EFAE6E30B02}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="0" windowHeight="0" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -52,7 +57,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -131,7 +136,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Standaard" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -443,7 +448,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
     <col min="2" max="2" width="14" customWidth="1"/>
@@ -451,7 +456,7 @@
     <col min="4" max="4" width="82" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -463,12 +468,12 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="45" customHeight="1">
+    <row r="2" spans="1:4" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>3</v>
       </c>
       <c r="B2" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C2" s="4"/>
       <c r="D2" s="5" t="s">

</xml_diff>

<commit_message>
Test succes, back to round 1
</commit_message>
<xml_diff>
--- a/QuizSettings.xlsx
+++ b/QuizSettings.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cafnzholding-my.sharepoint.com/personal/thom_van_dusschoten_synerlogic_nl/Documents/Documenten/GitHub/Sustainability-quiz/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="8_{6C329D2D-B3E9-4563-A84D-2DB2372B69CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{084077E7-7CBA-4869-8D62-5EFAE6E30B02}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="8_{6C329D2D-B3E9-4563-A84D-2DB2372B69CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0B8F408F-D371-4D65-8267-CA6EC40C1299}"/>
   <bookViews>
     <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -473,7 +473,7 @@
         <v>3</v>
       </c>
       <c r="B2" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C2" s="4"/>
       <c r="D2" s="5" t="s">

</xml_diff>